<commit_message>
Refactored framework with DriverSetup and modular utilities
</commit_message>
<xml_diff>
--- a/bin/Debug/net8.0/TestData/EmployeeData.xlsx
+++ b/bin/Debug/net8.0/TestData/EmployeeData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\IC_Projects\Excersise\OrangeHRMHybridAutomationFramework\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7505CDD-49FE-4A98-B97E-C13B90651EF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52CDBC12-3EAF-4092-891F-C583DBF89B3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -392,7 +392,7 @@
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -420,7 +420,7 @@
         <v>2</v>
       </c>
       <c r="D2" s="1">
-        <v>102938470</v>
+        <v>10234</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -434,7 +434,7 @@
         <v>5</v>
       </c>
       <c r="D3" s="1">
-        <v>102938471</v>
+        <v>10235</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -448,7 +448,7 @@
         <v>8</v>
       </c>
       <c r="D4">
-        <v>10293842</v>
+        <v>10231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>